<commit_message>
bando de dados ajustado
Tirei o "=" que estava em alguns índices
</commit_message>
<xml_diff>
--- a/src/main/resources/indices/indices.xlsx
+++ b/src/main/resources/indices/indices.xlsx
@@ -54,7 +54,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm"/>
-    <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -128,10 +128,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4236,7 +4236,6 @@
         <v>45017</v>
       </c>
       <c r="C347" s="6">
-        <f>0.57</f>
         <v>0.56999999999999995</v>
       </c>
     </row>
@@ -4325,7 +4324,6 @@
         <v>45261</v>
       </c>
       <c r="C355" s="6">
-        <f>0.4</f>
         <v>0.4</v>
       </c>
     </row>
@@ -4348,7 +4346,6 @@
         <v>45323</v>
       </c>
       <c r="C357" s="6">
-        <f>0.78</f>
         <v>0.78</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Autor e Réu não são mais obrigatórios. Índices atualizados até 06/2026
</commit_message>
<xml_diff>
--- a/src/main/resources/indices/indices.xlsx
+++ b/src/main/resources/indices/indices.xlsx
@@ -8889,7 +8889,7 @@
         <v>46174</v>
       </c>
       <c r="C770" s="6">
-        <v>0</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="771" spans="1:3" x14ac:dyDescent="0.25">
@@ -21517,7 +21517,7 @@
         <v>46174</v>
       </c>
       <c r="C1918" s="6">
-        <v>0</v>
+        <v>1.1200000000000001</v>
       </c>
     </row>
     <row r="1919" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>